<commit_message>
Sync with user-updated template: Simplified border logic to prioritize direct cell borders while maintaining terminal-phase stability
</commit_message>
<xml_diff>
--- a/public/templates/overtime_template.xlsx
+++ b/public/templates/overtime_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\wordtoexcel\staff_manager\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A5C956-9E7A-462D-833B-2A9C02706444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC0B5D1-ABDD-438E-BABB-40293849311B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1305" yWindow="930" windowWidth="26265" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
+    <workbookView xWindow="6120" yWindow="1065" windowWidth="27150" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
   </bookViews>
   <sheets>
     <sheet name="0" sheetId="1" r:id="rId1"/>
@@ -336,7 +336,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -495,19 +495,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -728,26 +715,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -760,7 +734,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
@@ -778,176 +752,170 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1312,104 +1280,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
     </row>
     <row r="2" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="18" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="31" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="42"/>
-      <c r="G2" s="43"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="22"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="41" t="s">
+      <c r="I2" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="47"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="50" t="s">
+      <c r="J2" s="26"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="41" t="s">
+      <c r="M2" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="47"/>
-      <c r="O2" s="48"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="27"/>
     </row>
     <row r="3" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40"/>
+      <c r="A3" s="19"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="53"/>
+      <c r="C3" s="32"/>
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="46"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="25"/>
       <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="44"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="49"/>
-      <c r="L3" s="51"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="45"/>
-      <c r="O3" s="49"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="28"/>
     </row>
     <row r="4" spans="1:15" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="56" t="s">
+      <c r="B4" s="38"/>
+      <c r="C4" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="57"/>
-      <c r="E4" s="58" t="s">
+      <c r="D4" s="41"/>
+      <c r="E4" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="59"/>
+      <c r="F4" s="40"/>
       <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="55" t="s">
+      <c r="H4" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="60"/>
-      <c r="J4" s="61" t="s">
+      <c r="I4" s="41"/>
+      <c r="J4" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="62"/>
+      <c r="K4" s="43"/>
       <c r="L4" s="14" t="s">
         <v>14</v>
       </c>
@@ -1424,434 +1392,434 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="11"/>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="63" t="s">
+      <c r="D5" s="34"/>
+      <c r="E5" s="44" t="s">
         <v>25</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="30"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="65" t="s">
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="49" t="s">
         <v>25</v>
       </c>
       <c r="K5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="24" t="s">
+      <c r="L5" s="51" t="s">
         <v>23</v>
       </c>
       <c r="M5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="26"/>
-      <c r="O5" s="27"/>
+      <c r="N5" s="47"/>
+      <c r="O5" s="48"/>
     </row>
     <row r="6" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37"/>
+      <c r="A6" s="17"/>
       <c r="B6" s="11"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="64"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="45"/>
       <c r="F6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="30"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="66"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="50"/>
       <c r="K6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="25"/>
+      <c r="L6" s="52"/>
       <c r="M6" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="N6" s="26"/>
-      <c r="O6" s="27"/>
+      <c r="N6" s="47"/>
+      <c r="O6" s="48"/>
     </row>
     <row r="7" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="36"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="28"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="53"/>
       <c r="F7" s="12"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="22"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="57"/>
+      <c r="J7" s="58"/>
       <c r="K7" s="15"/>
-      <c r="L7" s="24"/>
+      <c r="L7" s="51"/>
       <c r="M7" s="13"/>
-      <c r="N7" s="34"/>
-      <c r="O7" s="35"/>
+      <c r="N7" s="56"/>
+      <c r="O7" s="57"/>
     </row>
     <row r="8" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="37"/>
-      <c r="B8" s="37"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="29"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="54"/>
       <c r="F8" s="12"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="23"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="57"/>
+      <c r="J8" s="59"/>
       <c r="K8" s="15"/>
-      <c r="L8" s="25"/>
+      <c r="L8" s="52"/>
       <c r="M8" s="13"/>
-      <c r="N8" s="34"/>
-      <c r="O8" s="35"/>
+      <c r="N8" s="56"/>
+      <c r="O8" s="57"/>
     </row>
     <row r="9" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="28"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="53"/>
       <c r="F9" s="12"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="22"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="47"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="58"/>
       <c r="K9" s="15"/>
-      <c r="L9" s="24"/>
+      <c r="L9" s="51"/>
       <c r="M9" s="13"/>
-      <c r="N9" s="26"/>
-      <c r="O9" s="27"/>
+      <c r="N9" s="47"/>
+      <c r="O9" s="48"/>
     </row>
     <row r="10" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="37"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="29"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="54"/>
       <c r="F10" s="12"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="23"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="59"/>
       <c r="K10" s="15"/>
-      <c r="L10" s="25"/>
+      <c r="L10" s="52"/>
       <c r="M10" s="13"/>
-      <c r="N10" s="26"/>
-      <c r="O10" s="27"/>
+      <c r="N10" s="47"/>
+      <c r="O10" s="48"/>
     </row>
     <row r="11" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="36"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="28"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="53"/>
       <c r="F11" s="12"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="22"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="58"/>
       <c r="K11" s="15"/>
-      <c r="L11" s="24"/>
+      <c r="L11" s="51"/>
       <c r="M11" s="13"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="27"/>
+      <c r="N11" s="47"/>
+      <c r="O11" s="48"/>
     </row>
     <row r="12" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="37"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="29"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="54"/>
       <c r="F12" s="12"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="23"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="59"/>
       <c r="K12" s="15"/>
-      <c r="L12" s="25"/>
+      <c r="L12" s="52"/>
       <c r="M12" s="13"/>
-      <c r="N12" s="26"/>
-      <c r="O12" s="27"/>
+      <c r="N12" s="47"/>
+      <c r="O12" s="48"/>
     </row>
     <row r="13" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="36"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="28"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="53"/>
       <c r="F13" s="12"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="22"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="47"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="58"/>
       <c r="K13" s="15"/>
-      <c r="L13" s="24"/>
+      <c r="L13" s="51"/>
       <c r="M13" s="13"/>
-      <c r="N13" s="26"/>
-      <c r="O13" s="27"/>
+      <c r="N13" s="47"/>
+      <c r="O13" s="48"/>
     </row>
     <row r="14" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="37"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="29"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="54"/>
       <c r="F14" s="12"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="23"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="59"/>
       <c r="K14" s="15"/>
-      <c r="L14" s="25"/>
+      <c r="L14" s="52"/>
       <c r="M14" s="13"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="27"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="48"/>
     </row>
     <row r="15" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="36"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="28"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="53"/>
       <c r="F15" s="12"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="22"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="48"/>
+      <c r="J15" s="58"/>
       <c r="K15" s="15"/>
-      <c r="L15" s="24"/>
+      <c r="L15" s="51"/>
       <c r="M15" s="13"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="27"/>
+      <c r="N15" s="47"/>
+      <c r="O15" s="48"/>
     </row>
     <row r="16" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="37"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="29"/>
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="54"/>
       <c r="F16" s="12"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="23"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="47"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="59"/>
       <c r="K16" s="15"/>
-      <c r="L16" s="25"/>
+      <c r="L16" s="52"/>
       <c r="M16" s="13"/>
-      <c r="N16" s="26"/>
-      <c r="O16" s="27"/>
+      <c r="N16" s="47"/>
+      <c r="O16" s="48"/>
     </row>
     <row r="17" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="36"/>
-      <c r="B17" s="36"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="28"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="53"/>
       <c r="F17" s="12"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="22"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="47"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="58"/>
       <c r="K17" s="15"/>
-      <c r="L17" s="24"/>
+      <c r="L17" s="51"/>
       <c r="M17" s="13"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="27"/>
+      <c r="N17" s="47"/>
+      <c r="O17" s="48"/>
     </row>
     <row r="18" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="37"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="29"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="54"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="23"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="47"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="59"/>
       <c r="K18" s="15"/>
-      <c r="L18" s="25"/>
+      <c r="L18" s="52"/>
       <c r="M18" s="13"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="27"/>
+      <c r="N18" s="47"/>
+      <c r="O18" s="48"/>
     </row>
     <row r="19" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="36"/>
-      <c r="B19" s="36"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="28"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="53"/>
       <c r="F19" s="12"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="22"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="58"/>
       <c r="K19" s="15"/>
-      <c r="L19" s="24"/>
+      <c r="L19" s="51"/>
       <c r="M19" s="13"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="27"/>
+      <c r="N19" s="47"/>
+      <c r="O19" s="48"/>
     </row>
     <row r="20" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="37"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="29"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="54"/>
       <c r="F20" s="12"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="23"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="47"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="59"/>
       <c r="K20" s="15"/>
-      <c r="L20" s="25"/>
+      <c r="L20" s="52"/>
       <c r="M20" s="13"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="27"/>
+      <c r="N20" s="47"/>
+      <c r="O20" s="48"/>
     </row>
     <row r="21" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="36"/>
-      <c r="B21" s="36"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="28"/>
+      <c r="A21" s="16"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="53"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="22"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="47"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="58"/>
       <c r="K21" s="15"/>
-      <c r="L21" s="24"/>
+      <c r="L21" s="51"/>
       <c r="M21" s="13"/>
-      <c r="N21" s="26"/>
-      <c r="O21" s="27"/>
+      <c r="N21" s="47"/>
+      <c r="O21" s="48"/>
     </row>
     <row r="22" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="37"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="29"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="54"/>
       <c r="F22" s="12"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="23"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="59"/>
       <c r="K22" s="15"/>
-      <c r="L22" s="25"/>
+      <c r="L22" s="52"/>
       <c r="M22" s="13"/>
-      <c r="N22" s="26"/>
-      <c r="O22" s="27"/>
+      <c r="N22" s="47"/>
+      <c r="O22" s="48"/>
     </row>
     <row r="23" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="36"/>
-      <c r="B23" s="36"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="28"/>
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="53"/>
       <c r="F23" s="12"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="22"/>
+      <c r="G23" s="55"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="57"/>
+      <c r="J23" s="58"/>
       <c r="K23" s="15"/>
-      <c r="L23" s="24"/>
+      <c r="L23" s="51"/>
       <c r="M23" s="13"/>
-      <c r="N23" s="34"/>
-      <c r="O23" s="35"/>
+      <c r="N23" s="56"/>
+      <c r="O23" s="57"/>
     </row>
     <row r="24" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="37"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="29"/>
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="54"/>
       <c r="F24" s="12"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="23"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="57"/>
+      <c r="J24" s="59"/>
       <c r="K24" s="15"/>
-      <c r="L24" s="25"/>
+      <c r="L24" s="52"/>
       <c r="M24" s="13"/>
-      <c r="N24" s="34"/>
-      <c r="O24" s="35"/>
+      <c r="N24" s="56"/>
+      <c r="O24" s="57"/>
     </row>
     <row r="25" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="36"/>
-      <c r="B25" s="36"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="28"/>
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="53"/>
       <c r="F25" s="12"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="22"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="58"/>
       <c r="K25" s="15"/>
-      <c r="L25" s="24"/>
+      <c r="L25" s="51"/>
       <c r="M25" s="13"/>
-      <c r="N25" s="26"/>
-      <c r="O25" s="27"/>
+      <c r="N25" s="47"/>
+      <c r="O25" s="48"/>
     </row>
     <row r="26" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="37"/>
-      <c r="B26" s="37"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="29"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="54"/>
       <c r="F26" s="12"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="23"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="59"/>
       <c r="K26" s="15"/>
-      <c r="L26" s="25"/>
+      <c r="L26" s="52"/>
       <c r="M26" s="13"/>
-      <c r="N26" s="26"/>
-      <c r="O26" s="27"/>
+      <c r="N26" s="47"/>
+      <c r="O26" s="48"/>
     </row>
     <row r="27" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="36"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="28"/>
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="53"/>
       <c r="F27" s="12"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="27"/>
-      <c r="J27" s="22"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="47"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="58"/>
       <c r="K27" s="15"/>
-      <c r="L27" s="24"/>
+      <c r="L27" s="51"/>
       <c r="M27" s="13"/>
-      <c r="N27" s="26"/>
-      <c r="O27" s="27"/>
+      <c r="N27" s="47"/>
+      <c r="O27" s="48"/>
     </row>
     <row r="28" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="37"/>
-      <c r="B28" s="37"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="29"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="54"/>
       <c r="F28" s="12"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="23"/>
+      <c r="G28" s="64"/>
+      <c r="H28" s="60"/>
+      <c r="I28" s="61"/>
+      <c r="J28" s="59"/>
       <c r="K28" s="15"/>
-      <c r="L28" s="25"/>
+      <c r="L28" s="52"/>
       <c r="M28" s="13"/>
-      <c r="N28" s="32"/>
-      <c r="O28" s="33"/>
+      <c r="N28" s="60"/>
+      <c r="O28" s="61"/>
     </row>
     <row r="29" spans="1:15" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
@@ -1865,6 +1833,113 @@
     </row>
   </sheetData>
   <mergeCells count="131">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="C27:D28"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="N25:N26"/>
+    <mergeCell ref="O25:O26"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:I28"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="N23:N24"/>
+    <mergeCell ref="O23:O24"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:I26"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="N21:N22"/>
+    <mergeCell ref="O21:O22"/>
+    <mergeCell ref="C25:D26"/>
+    <mergeCell ref="C21:D22"/>
+    <mergeCell ref="C19:D20"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:I24"/>
+    <mergeCell ref="C23:D24"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:I20"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="C17:D18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:I16"/>
+    <mergeCell ref="C15:D16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="O15:O16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:I14"/>
+    <mergeCell ref="C13:D14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:I12"/>
+    <mergeCell ref="C11:D12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:I10"/>
+    <mergeCell ref="C9:D10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="A27:A28"/>
@@ -1889,113 +1964,6 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="O5:O6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="H7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:I10"/>
-    <mergeCell ref="C9:D10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:I12"/>
-    <mergeCell ref="C11:D12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:I14"/>
-    <mergeCell ref="C13:D14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:I16"/>
-    <mergeCell ref="C15:D16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="O15:O16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="C17:D18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:I20"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:I24"/>
-    <mergeCell ref="C23:D24"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="C27:D28"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="N25:N26"/>
-    <mergeCell ref="O25:O26"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:I28"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="N23:N24"/>
-    <mergeCell ref="O23:O24"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:I26"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="N21:N22"/>
-    <mergeCell ref="O21:O22"/>
-    <mergeCell ref="C25:D26"/>
-    <mergeCell ref="C21:D22"/>
-    <mergeCell ref="C19:D20"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
fix(export): remove code-side padding, delegate spacing to Excel template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/overtime_template.xlsx
+++ b/public/templates/overtime_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\wordtoexcel\staff_manager\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\dev\projects\wordtoexcel\staff_manager\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC0B5D1-ABDD-438E-BABB-40293849311B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F0A169-E6B8-4708-95AD-F1921A304D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6120" yWindow="1065" windowWidth="27150" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
+    <workbookView xWindow="1470" yWindow="1470" windowWidth="28455" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
   </bookViews>
   <sheets>
     <sheet name="0" sheetId="1" r:id="rId1"/>
@@ -202,11 +202,11 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>{{pay_check_n}}加班費 {{pay_hours_n}} 時</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>{{rest_check_n}}補休 {{rest_hours_n}} 時</t>
+    <t>{{rest_check_n}}補休{{rest_hours_n}}時</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{pay_check_n}}加班費 {{pay_hours_n}}時</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -770,10 +770,73 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="176" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -821,31 +884,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -860,62 +911,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1280,104 +1280,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
     </row>
     <row r="2" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="52" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="G2" s="22"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="43"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="26"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="29" t="s">
+      <c r="J2" s="47"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="20" t="s">
+      <c r="M2" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="26"/>
-      <c r="O2" s="27"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="48"/>
     </row>
     <row r="3" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
+      <c r="A3" s="40"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="32"/>
+      <c r="C3" s="53"/>
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="23"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="25"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="46"/>
       <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="23"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="28"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="45"/>
+      <c r="O3" s="49"/>
     </row>
     <row r="4" spans="1:15" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38" t="s">
+      <c r="B4" s="55"/>
+      <c r="C4" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="41"/>
-      <c r="E4" s="39" t="s">
+      <c r="D4" s="56"/>
+      <c r="E4" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="40"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="H4" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="41"/>
-      <c r="J4" s="42" t="s">
+      <c r="I4" s="56"/>
+      <c r="J4" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="43"/>
+      <c r="K4" s="60"/>
       <c r="L4" s="14" t="s">
         <v>14</v>
       </c>
@@ -1392,434 +1392,434 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="36" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="11"/>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="44" t="s">
+      <c r="D5" s="19"/>
+      <c r="E5" s="61" t="s">
         <v>25</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="46"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="49" t="s">
+      <c r="G5" s="30"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="63" t="s">
         <v>25</v>
       </c>
       <c r="K5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="51" t="s">
+      <c r="L5" s="24" t="s">
         <v>23</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="47"/>
-      <c r="O5" s="48"/>
+        <v>28</v>
+      </c>
+      <c r="N5" s="26"/>
+      <c r="O5" s="27"/>
     </row>
     <row r="6" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
+      <c r="A6" s="37"/>
       <c r="B6" s="11"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="45"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="62"/>
       <c r="F6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="46"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="50"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="64"/>
       <c r="K6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="52"/>
+      <c r="L6" s="25"/>
       <c r="M6" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="N6" s="47"/>
-      <c r="O6" s="48"/>
+        <v>27</v>
+      </c>
+      <c r="N6" s="26"/>
+      <c r="O6" s="27"/>
     </row>
     <row r="7" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="53"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="28"/>
       <c r="F7" s="12"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="57"/>
-      <c r="J7" s="58"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="22"/>
       <c r="K7" s="15"/>
-      <c r="L7" s="51"/>
+      <c r="L7" s="24"/>
       <c r="M7" s="13"/>
-      <c r="N7" s="56"/>
-      <c r="O7" s="57"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="35"/>
     </row>
     <row r="8" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="54"/>
+      <c r="A8" s="37"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="29"/>
       <c r="F8" s="12"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="57"/>
-      <c r="J8" s="59"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="23"/>
       <c r="K8" s="15"/>
-      <c r="L8" s="52"/>
+      <c r="L8" s="25"/>
       <c r="M8" s="13"/>
-      <c r="N8" s="56"/>
-      <c r="O8" s="57"/>
+      <c r="N8" s="34"/>
+      <c r="O8" s="35"/>
     </row>
     <row r="9" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="53"/>
+      <c r="A9" s="36"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="28"/>
       <c r="F9" s="12"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="47"/>
-      <c r="I9" s="48"/>
-      <c r="J9" s="58"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="22"/>
       <c r="K9" s="15"/>
-      <c r="L9" s="51"/>
+      <c r="L9" s="24"/>
       <c r="M9" s="13"/>
-      <c r="N9" s="47"/>
-      <c r="O9" s="48"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="27"/>
     </row>
     <row r="10" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="54"/>
+      <c r="A10" s="37"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="29"/>
       <c r="F10" s="12"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="59"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="23"/>
       <c r="K10" s="15"/>
-      <c r="L10" s="52"/>
+      <c r="L10" s="25"/>
       <c r="M10" s="13"/>
-      <c r="N10" s="47"/>
-      <c r="O10" s="48"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="27"/>
     </row>
     <row r="11" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="53"/>
+      <c r="A11" s="36"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="28"/>
       <c r="F11" s="12"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="48"/>
-      <c r="J11" s="58"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="22"/>
       <c r="K11" s="15"/>
-      <c r="L11" s="51"/>
+      <c r="L11" s="24"/>
       <c r="M11" s="13"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="48"/>
+      <c r="N11" s="26"/>
+      <c r="O11" s="27"/>
     </row>
     <row r="12" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="54"/>
+      <c r="A12" s="37"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="29"/>
       <c r="F12" s="12"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="48"/>
-      <c r="J12" s="59"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="23"/>
       <c r="K12" s="15"/>
-      <c r="L12" s="52"/>
+      <c r="L12" s="25"/>
       <c r="M12" s="13"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="48"/>
+      <c r="N12" s="26"/>
+      <c r="O12" s="27"/>
     </row>
     <row r="13" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="53"/>
+      <c r="A13" s="36"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="28"/>
       <c r="F13" s="12"/>
-      <c r="G13" s="46"/>
-      <c r="H13" s="47"/>
-      <c r="I13" s="48"/>
-      <c r="J13" s="58"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="22"/>
       <c r="K13" s="15"/>
-      <c r="L13" s="51"/>
+      <c r="L13" s="24"/>
       <c r="M13" s="13"/>
-      <c r="N13" s="47"/>
-      <c r="O13" s="48"/>
+      <c r="N13" s="26"/>
+      <c r="O13" s="27"/>
     </row>
     <row r="14" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="54"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="29"/>
       <c r="F14" s="12"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="59"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="23"/>
       <c r="K14" s="15"/>
-      <c r="L14" s="52"/>
+      <c r="L14" s="25"/>
       <c r="M14" s="13"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="48"/>
+      <c r="N14" s="26"/>
+      <c r="O14" s="27"/>
     </row>
     <row r="15" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="53"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="28"/>
       <c r="F15" s="12"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47"/>
-      <c r="I15" s="48"/>
-      <c r="J15" s="58"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="22"/>
       <c r="K15" s="15"/>
-      <c r="L15" s="51"/>
+      <c r="L15" s="24"/>
       <c r="M15" s="13"/>
-      <c r="N15" s="47"/>
-      <c r="O15" s="48"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="27"/>
     </row>
     <row r="16" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="54"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="29"/>
       <c r="F16" s="12"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="48"/>
-      <c r="J16" s="59"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="23"/>
       <c r="K16" s="15"/>
-      <c r="L16" s="52"/>
+      <c r="L16" s="25"/>
       <c r="M16" s="13"/>
-      <c r="N16" s="47"/>
-      <c r="O16" s="48"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="27"/>
     </row>
     <row r="17" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="53"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="28"/>
       <c r="F17" s="12"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="47"/>
-      <c r="I17" s="48"/>
-      <c r="J17" s="58"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="22"/>
       <c r="K17" s="15"/>
-      <c r="L17" s="51"/>
+      <c r="L17" s="24"/>
       <c r="M17" s="13"/>
-      <c r="N17" s="47"/>
-      <c r="O17" s="48"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="27"/>
     </row>
     <row r="18" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="54"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="29"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="47"/>
-      <c r="I18" s="48"/>
-      <c r="J18" s="59"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="23"/>
       <c r="K18" s="15"/>
-      <c r="L18" s="52"/>
+      <c r="L18" s="25"/>
       <c r="M18" s="13"/>
-      <c r="N18" s="47"/>
-      <c r="O18" s="48"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="27"/>
     </row>
     <row r="19" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="53"/>
+      <c r="A19" s="36"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="28"/>
       <c r="F19" s="12"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="47"/>
-      <c r="I19" s="48"/>
-      <c r="J19" s="58"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="22"/>
       <c r="K19" s="15"/>
-      <c r="L19" s="51"/>
+      <c r="L19" s="24"/>
       <c r="M19" s="13"/>
-      <c r="N19" s="47"/>
-      <c r="O19" s="48"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="27"/>
     </row>
     <row r="20" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="54"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="29"/>
       <c r="F20" s="12"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="47"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="59"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="23"/>
       <c r="K20" s="15"/>
-      <c r="L20" s="52"/>
+      <c r="L20" s="25"/>
       <c r="M20" s="13"/>
-      <c r="N20" s="47"/>
-      <c r="O20" s="48"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="27"/>
     </row>
     <row r="21" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="53"/>
+      <c r="A21" s="36"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="28"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="46"/>
-      <c r="H21" s="47"/>
-      <c r="I21" s="48"/>
-      <c r="J21" s="58"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="22"/>
       <c r="K21" s="15"/>
-      <c r="L21" s="51"/>
+      <c r="L21" s="24"/>
       <c r="M21" s="13"/>
-      <c r="N21" s="47"/>
-      <c r="O21" s="48"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="27"/>
     </row>
     <row r="22" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="54"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="29"/>
       <c r="F22" s="12"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="48"/>
-      <c r="J22" s="59"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="23"/>
       <c r="K22" s="15"/>
-      <c r="L22" s="52"/>
+      <c r="L22" s="25"/>
       <c r="M22" s="13"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="48"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="27"/>
     </row>
     <row r="23" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="53"/>
+      <c r="A23" s="36"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="28"/>
       <c r="F23" s="12"/>
-      <c r="G23" s="55"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="58"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="22"/>
       <c r="K23" s="15"/>
-      <c r="L23" s="51"/>
+      <c r="L23" s="24"/>
       <c r="M23" s="13"/>
-      <c r="N23" s="56"/>
-      <c r="O23" s="57"/>
+      <c r="N23" s="34"/>
+      <c r="O23" s="35"/>
     </row>
     <row r="24" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="17"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="54"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="29"/>
       <c r="F24" s="12"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="59"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="23"/>
       <c r="K24" s="15"/>
-      <c r="L24" s="52"/>
+      <c r="L24" s="25"/>
       <c r="M24" s="13"/>
-      <c r="N24" s="56"/>
-      <c r="O24" s="57"/>
+      <c r="N24" s="34"/>
+      <c r="O24" s="35"/>
     </row>
     <row r="25" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="53"/>
+      <c r="A25" s="36"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="28"/>
       <c r="F25" s="12"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="47"/>
-      <c r="I25" s="48"/>
-      <c r="J25" s="58"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="22"/>
       <c r="K25" s="15"/>
-      <c r="L25" s="51"/>
+      <c r="L25" s="24"/>
       <c r="M25" s="13"/>
-      <c r="N25" s="47"/>
-      <c r="O25" s="48"/>
+      <c r="N25" s="26"/>
+      <c r="O25" s="27"/>
     </row>
     <row r="26" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="54"/>
+      <c r="A26" s="37"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="29"/>
       <c r="F26" s="12"/>
-      <c r="G26" s="46"/>
-      <c r="H26" s="47"/>
-      <c r="I26" s="48"/>
-      <c r="J26" s="59"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="23"/>
       <c r="K26" s="15"/>
-      <c r="L26" s="52"/>
+      <c r="L26" s="25"/>
       <c r="M26" s="13"/>
-      <c r="N26" s="47"/>
-      <c r="O26" s="48"/>
+      <c r="N26" s="26"/>
+      <c r="O26" s="27"/>
     </row>
     <row r="27" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="53"/>
+      <c r="A27" s="36"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="28"/>
       <c r="F27" s="12"/>
-      <c r="G27" s="46"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="58"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="22"/>
       <c r="K27" s="15"/>
-      <c r="L27" s="51"/>
+      <c r="L27" s="24"/>
       <c r="M27" s="13"/>
-      <c r="N27" s="47"/>
-      <c r="O27" s="48"/>
+      <c r="N27" s="26"/>
+      <c r="O27" s="27"/>
     </row>
     <row r="28" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="54"/>
+      <c r="A28" s="37"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="29"/>
       <c r="F28" s="12"/>
-      <c r="G28" s="64"/>
-      <c r="H28" s="60"/>
-      <c r="I28" s="61"/>
-      <c r="J28" s="59"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="23"/>
       <c r="K28" s="15"/>
-      <c r="L28" s="52"/>
+      <c r="L28" s="25"/>
       <c r="M28" s="13"/>
-      <c r="N28" s="60"/>
-      <c r="O28" s="61"/>
+      <c r="N28" s="32"/>
+      <c r="O28" s="33"/>
     </row>
     <row r="29" spans="1:15" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
@@ -1833,6 +1833,113 @@
     </row>
   </sheetData>
   <mergeCells count="131">
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="E2:G3"/>
+    <mergeCell ref="I2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:O3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="C7:D8"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:I10"/>
+    <mergeCell ref="C9:D10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:I12"/>
+    <mergeCell ref="C11:D12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:I14"/>
+    <mergeCell ref="C13:D14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:I16"/>
+    <mergeCell ref="C15:D16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="O15:O16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="C17:D18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:I20"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:I24"/>
+    <mergeCell ref="C23:D24"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="C27:D28"/>
     <mergeCell ref="C5:D6"/>
@@ -1857,113 +1964,6 @@
     <mergeCell ref="C25:D26"/>
     <mergeCell ref="C21:D22"/>
     <mergeCell ref="C19:D20"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:I24"/>
-    <mergeCell ref="C23:D24"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:I20"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="C17:D18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:I16"/>
-    <mergeCell ref="C15:D16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="O15:O16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:I14"/>
-    <mergeCell ref="C13:D14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:I12"/>
-    <mergeCell ref="C11:D12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:I10"/>
-    <mergeCell ref="C9:D10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="H7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="E2:G3"/>
-    <mergeCell ref="I2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:O3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="C7:D8"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="O5:O6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
fix(export): remove rest_hours field and use template spacing; show build timestamp in sidebar
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/overtime_template.xlsx
+++ b/public/templates/overtime_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\dev\projects\wordtoexcel\staff_manager\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F0A169-E6B8-4708-95AD-F1921A304D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A90FA0-3FB3-4B25-BCEF-0EB285DCFFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="28455" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
+    <workbookView xWindow="2160" yWindow="2160" windowWidth="28455" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
   </bookViews>
   <sheets>
     <sheet name="0" sheetId="1" r:id="rId1"/>
@@ -202,11 +202,11 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>{{rest_check_n}}補休{{rest_hours_n}}時</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>{{pay_check_n}}加班費 {{pay_hours_n}}時</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>{{rest_check_n}}補休      時</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -770,152 +770,152 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1280,104 +1280,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
     </row>
     <row r="2" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="18" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="31" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="41" t="s">
+      <c r="E2" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="42"/>
-      <c r="G2" s="43"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="22"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="41" t="s">
+      <c r="I2" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="47"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="50" t="s">
+      <c r="J2" s="26"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="41" t="s">
+      <c r="M2" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="47"/>
-      <c r="O2" s="48"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="27"/>
     </row>
     <row r="3" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="40"/>
+      <c r="A3" s="19"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="53"/>
+      <c r="C3" s="32"/>
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="44"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="46"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="25"/>
       <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="44"/>
-      <c r="J3" s="45"/>
-      <c r="K3" s="49"/>
-      <c r="L3" s="51"/>
-      <c r="M3" s="44"/>
-      <c r="N3" s="45"/>
-      <c r="O3" s="49"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="28"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="28"/>
     </row>
     <row r="4" spans="1:15" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55" t="s">
+      <c r="B4" s="38"/>
+      <c r="C4" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="56"/>
-      <c r="E4" s="57" t="s">
+      <c r="D4" s="39"/>
+      <c r="E4" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="58"/>
+      <c r="F4" s="41"/>
       <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="55" t="s">
+      <c r="H4" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="56"/>
-      <c r="J4" s="59" t="s">
+      <c r="I4" s="39"/>
+      <c r="J4" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="60"/>
+      <c r="K4" s="43"/>
       <c r="L4" s="14" t="s">
         <v>14</v>
       </c>
@@ -1392,434 +1392,434 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="11"/>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="61" t="s">
+      <c r="D5" s="34"/>
+      <c r="E5" s="44" t="s">
         <v>25</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="30"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="63" t="s">
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="49" t="s">
         <v>25</v>
       </c>
       <c r="K5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="24" t="s">
+      <c r="L5" s="51" t="s">
         <v>23</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="N5" s="26"/>
-      <c r="O5" s="27"/>
+        <v>27</v>
+      </c>
+      <c r="N5" s="47"/>
+      <c r="O5" s="48"/>
     </row>
     <row r="6" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37"/>
+      <c r="A6" s="17"/>
       <c r="B6" s="11"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="62"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="45"/>
       <c r="F6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="30"/>
-      <c r="H6" s="26"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="64"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="47"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="50"/>
       <c r="K6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="25"/>
+      <c r="L6" s="52"/>
       <c r="M6" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="26"/>
-      <c r="O6" s="27"/>
+        <v>28</v>
+      </c>
+      <c r="N6" s="47"/>
+      <c r="O6" s="48"/>
     </row>
     <row r="7" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="36"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="28"/>
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="53"/>
       <c r="F7" s="12"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="22"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="56"/>
+      <c r="I7" s="57"/>
+      <c r="J7" s="58"/>
       <c r="K7" s="15"/>
-      <c r="L7" s="24"/>
+      <c r="L7" s="51"/>
       <c r="M7" s="13"/>
-      <c r="N7" s="34"/>
-      <c r="O7" s="35"/>
+      <c r="N7" s="56"/>
+      <c r="O7" s="57"/>
     </row>
     <row r="8" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="37"/>
-      <c r="B8" s="37"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="21"/>
-      <c r="E8" s="29"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="54"/>
       <c r="F8" s="12"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="23"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="56"/>
+      <c r="I8" s="57"/>
+      <c r="J8" s="59"/>
       <c r="K8" s="15"/>
-      <c r="L8" s="25"/>
+      <c r="L8" s="52"/>
       <c r="M8" s="13"/>
-      <c r="N8" s="34"/>
-      <c r="O8" s="35"/>
+      <c r="N8" s="56"/>
+      <c r="O8" s="57"/>
     </row>
     <row r="9" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="28"/>
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="53"/>
       <c r="F9" s="12"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="22"/>
+      <c r="G9" s="46"/>
+      <c r="H9" s="47"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="58"/>
       <c r="K9" s="15"/>
-      <c r="L9" s="24"/>
+      <c r="L9" s="51"/>
       <c r="M9" s="13"/>
-      <c r="N9" s="26"/>
-      <c r="O9" s="27"/>
+      <c r="N9" s="47"/>
+      <c r="O9" s="48"/>
     </row>
     <row r="10" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="37"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="29"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="36"/>
+      <c r="E10" s="54"/>
       <c r="F10" s="12"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="23"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="59"/>
       <c r="K10" s="15"/>
-      <c r="L10" s="25"/>
+      <c r="L10" s="52"/>
       <c r="M10" s="13"/>
-      <c r="N10" s="26"/>
-      <c r="O10" s="27"/>
+      <c r="N10" s="47"/>
+      <c r="O10" s="48"/>
     </row>
     <row r="11" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="36"/>
-      <c r="B11" s="36"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="28"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="53"/>
       <c r="F11" s="12"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="22"/>
+      <c r="G11" s="46"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="58"/>
       <c r="K11" s="15"/>
-      <c r="L11" s="24"/>
+      <c r="L11" s="51"/>
       <c r="M11" s="13"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="27"/>
+      <c r="N11" s="47"/>
+      <c r="O11" s="48"/>
     </row>
     <row r="12" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="37"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="29"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="54"/>
       <c r="F12" s="12"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="23"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="47"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="59"/>
       <c r="K12" s="15"/>
-      <c r="L12" s="25"/>
+      <c r="L12" s="52"/>
       <c r="M12" s="13"/>
-      <c r="N12" s="26"/>
-      <c r="O12" s="27"/>
+      <c r="N12" s="47"/>
+      <c r="O12" s="48"/>
     </row>
     <row r="13" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="36"/>
-      <c r="B13" s="36"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="28"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="53"/>
       <c r="F13" s="12"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="22"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="47"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="58"/>
       <c r="K13" s="15"/>
-      <c r="L13" s="24"/>
+      <c r="L13" s="51"/>
       <c r="M13" s="13"/>
-      <c r="N13" s="26"/>
-      <c r="O13" s="27"/>
+      <c r="N13" s="47"/>
+      <c r="O13" s="48"/>
     </row>
     <row r="14" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="37"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="29"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="54"/>
       <c r="F14" s="12"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="23"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="59"/>
       <c r="K14" s="15"/>
-      <c r="L14" s="25"/>
+      <c r="L14" s="52"/>
       <c r="M14" s="13"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="27"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="48"/>
     </row>
     <row r="15" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="36"/>
-      <c r="B15" s="36"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="28"/>
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="53"/>
       <c r="F15" s="12"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="22"/>
+      <c r="G15" s="46"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="48"/>
+      <c r="J15" s="58"/>
       <c r="K15" s="15"/>
-      <c r="L15" s="24"/>
+      <c r="L15" s="51"/>
       <c r="M15" s="13"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="27"/>
+      <c r="N15" s="47"/>
+      <c r="O15" s="48"/>
     </row>
     <row r="16" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="37"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="29"/>
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="54"/>
       <c r="F16" s="12"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="23"/>
+      <c r="G16" s="46"/>
+      <c r="H16" s="47"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="59"/>
       <c r="K16" s="15"/>
-      <c r="L16" s="25"/>
+      <c r="L16" s="52"/>
       <c r="M16" s="13"/>
-      <c r="N16" s="26"/>
-      <c r="O16" s="27"/>
+      <c r="N16" s="47"/>
+      <c r="O16" s="48"/>
     </row>
     <row r="17" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="36"/>
-      <c r="B17" s="36"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="28"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="53"/>
       <c r="F17" s="12"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="22"/>
+      <c r="G17" s="46"/>
+      <c r="H17" s="47"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="58"/>
       <c r="K17" s="15"/>
-      <c r="L17" s="24"/>
+      <c r="L17" s="51"/>
       <c r="M17" s="13"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="27"/>
+      <c r="N17" s="47"/>
+      <c r="O17" s="48"/>
     </row>
     <row r="18" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="37"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="29"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="54"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="23"/>
+      <c r="G18" s="46"/>
+      <c r="H18" s="47"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="59"/>
       <c r="K18" s="15"/>
-      <c r="L18" s="25"/>
+      <c r="L18" s="52"/>
       <c r="M18" s="13"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="27"/>
+      <c r="N18" s="47"/>
+      <c r="O18" s="48"/>
     </row>
     <row r="19" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="36"/>
-      <c r="B19" s="36"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="28"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="53"/>
       <c r="F19" s="12"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="22"/>
+      <c r="G19" s="46"/>
+      <c r="H19" s="47"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="58"/>
       <c r="K19" s="15"/>
-      <c r="L19" s="24"/>
+      <c r="L19" s="51"/>
       <c r="M19" s="13"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="27"/>
+      <c r="N19" s="47"/>
+      <c r="O19" s="48"/>
     </row>
     <row r="20" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="37"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="29"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="54"/>
       <c r="F20" s="12"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="23"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="47"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="59"/>
       <c r="K20" s="15"/>
-      <c r="L20" s="25"/>
+      <c r="L20" s="52"/>
       <c r="M20" s="13"/>
-      <c r="N20" s="26"/>
-      <c r="O20" s="27"/>
+      <c r="N20" s="47"/>
+      <c r="O20" s="48"/>
     </row>
     <row r="21" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="36"/>
-      <c r="B21" s="36"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="28"/>
+      <c r="A21" s="16"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="53"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="27"/>
-      <c r="J21" s="22"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="47"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="58"/>
       <c r="K21" s="15"/>
-      <c r="L21" s="24"/>
+      <c r="L21" s="51"/>
       <c r="M21" s="13"/>
-      <c r="N21" s="26"/>
-      <c r="O21" s="27"/>
+      <c r="N21" s="47"/>
+      <c r="O21" s="48"/>
     </row>
     <row r="22" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="37"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="29"/>
+      <c r="A22" s="17"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="54"/>
       <c r="F22" s="12"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="27"/>
-      <c r="J22" s="23"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="47"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="59"/>
       <c r="K22" s="15"/>
-      <c r="L22" s="25"/>
+      <c r="L22" s="52"/>
       <c r="M22" s="13"/>
-      <c r="N22" s="26"/>
-      <c r="O22" s="27"/>
+      <c r="N22" s="47"/>
+      <c r="O22" s="48"/>
     </row>
     <row r="23" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="36"/>
-      <c r="B23" s="36"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="28"/>
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="53"/>
       <c r="F23" s="12"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="22"/>
+      <c r="G23" s="55"/>
+      <c r="H23" s="56"/>
+      <c r="I23" s="57"/>
+      <c r="J23" s="58"/>
       <c r="K23" s="15"/>
-      <c r="L23" s="24"/>
+      <c r="L23" s="51"/>
       <c r="M23" s="13"/>
-      <c r="N23" s="34"/>
-      <c r="O23" s="35"/>
+      <c r="N23" s="56"/>
+      <c r="O23" s="57"/>
     </row>
     <row r="24" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="37"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="29"/>
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="54"/>
       <c r="F24" s="12"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="23"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="57"/>
+      <c r="J24" s="59"/>
       <c r="K24" s="15"/>
-      <c r="L24" s="25"/>
+      <c r="L24" s="52"/>
       <c r="M24" s="13"/>
-      <c r="N24" s="34"/>
-      <c r="O24" s="35"/>
+      <c r="N24" s="56"/>
+      <c r="O24" s="57"/>
     </row>
     <row r="25" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="36"/>
-      <c r="B25" s="36"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="28"/>
+      <c r="A25" s="16"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="53"/>
       <c r="F25" s="12"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="22"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="58"/>
       <c r="K25" s="15"/>
-      <c r="L25" s="24"/>
+      <c r="L25" s="51"/>
       <c r="M25" s="13"/>
-      <c r="N25" s="26"/>
-      <c r="O25" s="27"/>
+      <c r="N25" s="47"/>
+      <c r="O25" s="48"/>
     </row>
     <row r="26" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="37"/>
-      <c r="B26" s="37"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="29"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="35"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="54"/>
       <c r="F26" s="12"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="23"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="47"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="59"/>
       <c r="K26" s="15"/>
-      <c r="L26" s="25"/>
+      <c r="L26" s="52"/>
       <c r="M26" s="13"/>
-      <c r="N26" s="26"/>
-      <c r="O26" s="27"/>
+      <c r="N26" s="47"/>
+      <c r="O26" s="48"/>
     </row>
     <row r="27" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="36"/>
-      <c r="B27" s="36"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="28"/>
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="53"/>
       <c r="F27" s="12"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="26"/>
-      <c r="I27" s="27"/>
-      <c r="J27" s="22"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="47"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="58"/>
       <c r="K27" s="15"/>
-      <c r="L27" s="24"/>
+      <c r="L27" s="51"/>
       <c r="M27" s="13"/>
-      <c r="N27" s="26"/>
-      <c r="O27" s="27"/>
+      <c r="N27" s="47"/>
+      <c r="O27" s="48"/>
     </row>
     <row r="28" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="37"/>
-      <c r="B28" s="37"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="29"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="36"/>
+      <c r="E28" s="54"/>
       <c r="F28" s="12"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="23"/>
+      <c r="G28" s="64"/>
+      <c r="H28" s="60"/>
+      <c r="I28" s="61"/>
+      <c r="J28" s="59"/>
       <c r="K28" s="15"/>
-      <c r="L28" s="25"/>
+      <c r="L28" s="52"/>
       <c r="M28" s="13"/>
-      <c r="N28" s="32"/>
-      <c r="O28" s="33"/>
+      <c r="N28" s="60"/>
+      <c r="O28" s="61"/>
     </row>
     <row r="29" spans="1:15" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
@@ -1833,6 +1833,113 @@
     </row>
   </sheetData>
   <mergeCells count="131">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="C27:D28"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="N25:N26"/>
+    <mergeCell ref="O25:O26"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:I28"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="N23:N24"/>
+    <mergeCell ref="O23:O24"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:I26"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="N21:N22"/>
+    <mergeCell ref="O21:O22"/>
+    <mergeCell ref="C25:D26"/>
+    <mergeCell ref="C21:D22"/>
+    <mergeCell ref="C19:D20"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:I24"/>
+    <mergeCell ref="C23:D24"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:I20"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="C17:D18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:I16"/>
+    <mergeCell ref="C15:D16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="O15:O16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:I14"/>
+    <mergeCell ref="C13:D14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:I12"/>
+    <mergeCell ref="C11:D12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:I10"/>
+    <mergeCell ref="C9:D10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="A27:A28"/>
@@ -1857,113 +1964,6 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="O5:O6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="H7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:I10"/>
-    <mergeCell ref="C9:D10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:I12"/>
-    <mergeCell ref="C11:D12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:I14"/>
-    <mergeCell ref="C13:D14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:I16"/>
-    <mergeCell ref="C15:D16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="O15:O16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="C17:D18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:I20"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:I24"/>
-    <mergeCell ref="C23:D24"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="C27:D28"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="J25:J26"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="N25:N26"/>
-    <mergeCell ref="O25:O26"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="H27:I28"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="N23:N24"/>
-    <mergeCell ref="O23:O24"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:I26"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="N21:N22"/>
-    <mergeCell ref="O21:O22"/>
-    <mergeCell ref="C25:D26"/>
-    <mergeCell ref="C21:D22"/>
-    <mergeCell ref="C19:D20"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
fix(template): update overtime template spacing for pay/rest hours fields
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/overtime_template.xlsx
+++ b/public/templates/overtime_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\dev\projects\wordtoexcel\staff_manager\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55A90FA0-3FB3-4B25-BCEF-0EB285DCFFD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{096AEEDD-236E-419A-A7CB-845CF0377440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="28455" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
+    <workbookView xWindow="1440" yWindow="1365" windowWidth="28455" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
   </bookViews>
   <sheets>
     <sheet name="0" sheetId="1" r:id="rId1"/>
@@ -206,7 +206,7 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>{{rest_check_n}}補休      時</t>
+    <t>{{rest_check_n}}補休     時</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -770,10 +770,73 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="176" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -821,18 +884,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -860,62 +911,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1280,104 +1280,104 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
-      <c r="M1" s="63"/>
-      <c r="N1" s="63"/>
-      <c r="O1" s="63"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
     </row>
     <row r="2" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="52" t="s">
         <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="21"/>
-      <c r="G2" s="22"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="43"/>
       <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="26"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="29" t="s">
+      <c r="J2" s="47"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="20" t="s">
+      <c r="M2" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="N2" s="26"/>
-      <c r="O2" s="27"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="48"/>
     </row>
     <row r="3" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
+      <c r="A3" s="40"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="32"/>
+      <c r="C3" s="53"/>
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="23"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="25"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="46"/>
       <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="23"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="30"/>
-      <c r="M3" s="23"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="28"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="49"/>
+      <c r="L3" s="51"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="45"/>
+      <c r="O3" s="49"/>
     </row>
     <row r="4" spans="1:15" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="38" t="s">
+      <c r="B4" s="55"/>
+      <c r="C4" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="39"/>
-      <c r="E4" s="40" t="s">
+      <c r="D4" s="56"/>
+      <c r="E4" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="41"/>
+      <c r="F4" s="58"/>
       <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="H4" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="39"/>
-      <c r="J4" s="42" t="s">
+      <c r="I4" s="56"/>
+      <c r="J4" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="43"/>
+      <c r="K4" s="60"/>
       <c r="L4" s="14" t="s">
         <v>14</v>
       </c>
@@ -1392,434 +1392,434 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="36" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="11"/>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="44" t="s">
+      <c r="D5" s="19"/>
+      <c r="E5" s="61" t="s">
         <v>25</v>
       </c>
       <c r="F5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="46"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="49" t="s">
+      <c r="G5" s="30"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="63" t="s">
         <v>25</v>
       </c>
       <c r="K5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="51" t="s">
+      <c r="L5" s="24" t="s">
         <v>23</v>
       </c>
       <c r="M5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="47"/>
-      <c r="O5" s="48"/>
+      <c r="N5" s="26"/>
+      <c r="O5" s="27"/>
     </row>
     <row r="6" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
+      <c r="A6" s="37"/>
       <c r="B6" s="11"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="45"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="62"/>
       <c r="F6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="46"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="48"/>
-      <c r="J6" s="50"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="26"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="64"/>
       <c r="K6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="L6" s="52"/>
+      <c r="L6" s="25"/>
       <c r="M6" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="N6" s="47"/>
-      <c r="O6" s="48"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="27"/>
     </row>
     <row r="7" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="53"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="28"/>
       <c r="F7" s="12"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="57"/>
-      <c r="J7" s="58"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="22"/>
       <c r="K7" s="15"/>
-      <c r="L7" s="51"/>
+      <c r="L7" s="24"/>
       <c r="M7" s="13"/>
-      <c r="N7" s="56"/>
-      <c r="O7" s="57"/>
+      <c r="N7" s="34"/>
+      <c r="O7" s="35"/>
     </row>
     <row r="8" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="54"/>
+      <c r="A8" s="37"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="29"/>
       <c r="F8" s="12"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="56"/>
-      <c r="I8" s="57"/>
-      <c r="J8" s="59"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="23"/>
       <c r="K8" s="15"/>
-      <c r="L8" s="52"/>
+      <c r="L8" s="25"/>
       <c r="M8" s="13"/>
-      <c r="N8" s="56"/>
-      <c r="O8" s="57"/>
+      <c r="N8" s="34"/>
+      <c r="O8" s="35"/>
     </row>
     <row r="9" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="53"/>
+      <c r="A9" s="36"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="28"/>
       <c r="F9" s="12"/>
-      <c r="G9" s="46"/>
-      <c r="H9" s="47"/>
-      <c r="I9" s="48"/>
-      <c r="J9" s="58"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="22"/>
       <c r="K9" s="15"/>
-      <c r="L9" s="51"/>
+      <c r="L9" s="24"/>
       <c r="M9" s="13"/>
-      <c r="N9" s="47"/>
-      <c r="O9" s="48"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="27"/>
     </row>
     <row r="10" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="54"/>
+      <c r="A10" s="37"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="29"/>
       <c r="F10" s="12"/>
-      <c r="G10" s="46"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="59"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="26"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="23"/>
       <c r="K10" s="15"/>
-      <c r="L10" s="52"/>
+      <c r="L10" s="25"/>
       <c r="M10" s="13"/>
-      <c r="N10" s="47"/>
-      <c r="O10" s="48"/>
+      <c r="N10" s="26"/>
+      <c r="O10" s="27"/>
     </row>
     <row r="11" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="53"/>
+      <c r="A11" s="36"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="28"/>
       <c r="F11" s="12"/>
-      <c r="G11" s="46"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="48"/>
-      <c r="J11" s="58"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="22"/>
       <c r="K11" s="15"/>
-      <c r="L11" s="51"/>
+      <c r="L11" s="24"/>
       <c r="M11" s="13"/>
-      <c r="N11" s="47"/>
-      <c r="O11" s="48"/>
+      <c r="N11" s="26"/>
+      <c r="O11" s="27"/>
     </row>
     <row r="12" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="54"/>
+      <c r="A12" s="37"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="29"/>
       <c r="F12" s="12"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="47"/>
-      <c r="I12" s="48"/>
-      <c r="J12" s="59"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="23"/>
       <c r="K12" s="15"/>
-      <c r="L12" s="52"/>
+      <c r="L12" s="25"/>
       <c r="M12" s="13"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="48"/>
+      <c r="N12" s="26"/>
+      <c r="O12" s="27"/>
     </row>
     <row r="13" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="16"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="53"/>
+      <c r="A13" s="36"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="28"/>
       <c r="F13" s="12"/>
-      <c r="G13" s="46"/>
-      <c r="H13" s="47"/>
-      <c r="I13" s="48"/>
-      <c r="J13" s="58"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="22"/>
       <c r="K13" s="15"/>
-      <c r="L13" s="51"/>
+      <c r="L13" s="24"/>
       <c r="M13" s="13"/>
-      <c r="N13" s="47"/>
-      <c r="O13" s="48"/>
+      <c r="N13" s="26"/>
+      <c r="O13" s="27"/>
     </row>
     <row r="14" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="54"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="29"/>
       <c r="F14" s="12"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="47"/>
-      <c r="I14" s="48"/>
-      <c r="J14" s="59"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="23"/>
       <c r="K14" s="15"/>
-      <c r="L14" s="52"/>
+      <c r="L14" s="25"/>
       <c r="M14" s="13"/>
-      <c r="N14" s="47"/>
-      <c r="O14" s="48"/>
+      <c r="N14" s="26"/>
+      <c r="O14" s="27"/>
     </row>
     <row r="15" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="53"/>
+      <c r="A15" s="36"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="28"/>
       <c r="F15" s="12"/>
-      <c r="G15" s="46"/>
-      <c r="H15" s="47"/>
-      <c r="I15" s="48"/>
-      <c r="J15" s="58"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="22"/>
       <c r="K15" s="15"/>
-      <c r="L15" s="51"/>
+      <c r="L15" s="24"/>
       <c r="M15" s="13"/>
-      <c r="N15" s="47"/>
-      <c r="O15" s="48"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="27"/>
     </row>
     <row r="16" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="54"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="29"/>
       <c r="F16" s="12"/>
-      <c r="G16" s="46"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="48"/>
-      <c r="J16" s="59"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="23"/>
       <c r="K16" s="15"/>
-      <c r="L16" s="52"/>
+      <c r="L16" s="25"/>
       <c r="M16" s="13"/>
-      <c r="N16" s="47"/>
-      <c r="O16" s="48"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="27"/>
     </row>
     <row r="17" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="53"/>
+      <c r="A17" s="36"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="28"/>
       <c r="F17" s="12"/>
-      <c r="G17" s="46"/>
-      <c r="H17" s="47"/>
-      <c r="I17" s="48"/>
-      <c r="J17" s="58"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="22"/>
       <c r="K17" s="15"/>
-      <c r="L17" s="51"/>
+      <c r="L17" s="24"/>
       <c r="M17" s="13"/>
-      <c r="N17" s="47"/>
-      <c r="O17" s="48"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="27"/>
     </row>
     <row r="18" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="54"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="29"/>
       <c r="F18" s="12"/>
-      <c r="G18" s="46"/>
-      <c r="H18" s="47"/>
-      <c r="I18" s="48"/>
-      <c r="J18" s="59"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="23"/>
       <c r="K18" s="15"/>
-      <c r="L18" s="52"/>
+      <c r="L18" s="25"/>
       <c r="M18" s="13"/>
-      <c r="N18" s="47"/>
-      <c r="O18" s="48"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="27"/>
     </row>
     <row r="19" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="53"/>
+      <c r="A19" s="36"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="28"/>
       <c r="F19" s="12"/>
-      <c r="G19" s="46"/>
-      <c r="H19" s="47"/>
-      <c r="I19" s="48"/>
-      <c r="J19" s="58"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="22"/>
       <c r="K19" s="15"/>
-      <c r="L19" s="51"/>
+      <c r="L19" s="24"/>
       <c r="M19" s="13"/>
-      <c r="N19" s="47"/>
-      <c r="O19" s="48"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="27"/>
     </row>
     <row r="20" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="54"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="29"/>
       <c r="F20" s="12"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="47"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="59"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="23"/>
       <c r="K20" s="15"/>
-      <c r="L20" s="52"/>
+      <c r="L20" s="25"/>
       <c r="M20" s="13"/>
-      <c r="N20" s="47"/>
-      <c r="O20" s="48"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="27"/>
     </row>
     <row r="21" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="53"/>
+      <c r="A21" s="36"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="28"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="46"/>
-      <c r="H21" s="47"/>
-      <c r="I21" s="48"/>
-      <c r="J21" s="58"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="22"/>
       <c r="K21" s="15"/>
-      <c r="L21" s="51"/>
+      <c r="L21" s="24"/>
       <c r="M21" s="13"/>
-      <c r="N21" s="47"/>
-      <c r="O21" s="48"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="27"/>
     </row>
     <row r="22" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="54"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="29"/>
       <c r="F22" s="12"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="47"/>
-      <c r="I22" s="48"/>
-      <c r="J22" s="59"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="23"/>
       <c r="K22" s="15"/>
-      <c r="L22" s="52"/>
+      <c r="L22" s="25"/>
       <c r="M22" s="13"/>
-      <c r="N22" s="47"/>
-      <c r="O22" s="48"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="27"/>
     </row>
     <row r="23" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="53"/>
+      <c r="A23" s="36"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="28"/>
       <c r="F23" s="12"/>
-      <c r="G23" s="55"/>
-      <c r="H23" s="56"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="58"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="22"/>
       <c r="K23" s="15"/>
-      <c r="L23" s="51"/>
+      <c r="L23" s="24"/>
       <c r="M23" s="13"/>
-      <c r="N23" s="56"/>
-      <c r="O23" s="57"/>
+      <c r="N23" s="34"/>
+      <c r="O23" s="35"/>
     </row>
     <row r="24" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="17"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="54"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="29"/>
       <c r="F24" s="12"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="56"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="59"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="23"/>
       <c r="K24" s="15"/>
-      <c r="L24" s="52"/>
+      <c r="L24" s="25"/>
       <c r="M24" s="13"/>
-      <c r="N24" s="56"/>
-      <c r="O24" s="57"/>
+      <c r="N24" s="34"/>
+      <c r="O24" s="35"/>
     </row>
     <row r="25" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="53"/>
+      <c r="A25" s="36"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="28"/>
       <c r="F25" s="12"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="47"/>
-      <c r="I25" s="48"/>
-      <c r="J25" s="58"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="26"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="22"/>
       <c r="K25" s="15"/>
-      <c r="L25" s="51"/>
+      <c r="L25" s="24"/>
       <c r="M25" s="13"/>
-      <c r="N25" s="47"/>
-      <c r="O25" s="48"/>
+      <c r="N25" s="26"/>
+      <c r="O25" s="27"/>
     </row>
     <row r="26" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="35"/>
-      <c r="D26" s="36"/>
-      <c r="E26" s="54"/>
+      <c r="A26" s="37"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="29"/>
       <c r="F26" s="12"/>
-      <c r="G26" s="46"/>
-      <c r="H26" s="47"/>
-      <c r="I26" s="48"/>
-      <c r="J26" s="59"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="26"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="23"/>
       <c r="K26" s="15"/>
-      <c r="L26" s="52"/>
+      <c r="L26" s="25"/>
       <c r="M26" s="13"/>
-      <c r="N26" s="47"/>
-      <c r="O26" s="48"/>
+      <c r="N26" s="26"/>
+      <c r="O26" s="27"/>
     </row>
     <row r="27" spans="1:15" ht="25.35" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="53"/>
+      <c r="A27" s="36"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="28"/>
       <c r="F27" s="12"/>
-      <c r="G27" s="46"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="48"/>
-      <c r="J27" s="58"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="26"/>
+      <c r="I27" s="27"/>
+      <c r="J27" s="22"/>
       <c r="K27" s="15"/>
-      <c r="L27" s="51"/>
+      <c r="L27" s="24"/>
       <c r="M27" s="13"/>
-      <c r="N27" s="47"/>
-      <c r="O27" s="48"/>
+      <c r="N27" s="26"/>
+      <c r="O27" s="27"/>
     </row>
     <row r="28" spans="1:15" ht="25.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="35"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="54"/>
+      <c r="A28" s="37"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="29"/>
       <c r="F28" s="12"/>
-      <c r="G28" s="64"/>
-      <c r="H28" s="60"/>
-      <c r="I28" s="61"/>
-      <c r="J28" s="59"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="23"/>
       <c r="K28" s="15"/>
-      <c r="L28" s="52"/>
+      <c r="L28" s="25"/>
       <c r="M28" s="13"/>
-      <c r="N28" s="60"/>
-      <c r="O28" s="61"/>
+      <c r="N28" s="32"/>
+      <c r="O28" s="33"/>
     </row>
     <row r="29" spans="1:15" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
@@ -1833,6 +1833,113 @@
     </row>
   </sheetData>
   <mergeCells count="131">
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="E2:G3"/>
+    <mergeCell ref="I2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:O3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="C7:D8"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:I6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="L5:L6"/>
+    <mergeCell ref="N5:N6"/>
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H9:I10"/>
+    <mergeCell ref="C9:D10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H11:I12"/>
+    <mergeCell ref="C11:D12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:I14"/>
+    <mergeCell ref="C13:D14"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="N13:N14"/>
+    <mergeCell ref="O13:O14"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:I16"/>
+    <mergeCell ref="C15:D16"/>
+    <mergeCell ref="J15:J16"/>
+    <mergeCell ref="L15:L16"/>
+    <mergeCell ref="N15:N16"/>
+    <mergeCell ref="O15:O16"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="C17:D18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="N27:N28"/>
+    <mergeCell ref="O27:O28"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:I22"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:I20"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:I24"/>
+    <mergeCell ref="C23:D24"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="C27:D28"/>
     <mergeCell ref="C5:D6"/>
@@ -1857,113 +1964,6 @@
     <mergeCell ref="C25:D26"/>
     <mergeCell ref="C21:D22"/>
     <mergeCell ref="C19:D20"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:I24"/>
-    <mergeCell ref="C23:D24"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="N27:N28"/>
-    <mergeCell ref="O27:O28"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:I22"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:I20"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="C17:D18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:I16"/>
-    <mergeCell ref="C15:D16"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="L15:L16"/>
-    <mergeCell ref="N15:N16"/>
-    <mergeCell ref="O15:O16"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="H13:I14"/>
-    <mergeCell ref="C13:D14"/>
-    <mergeCell ref="J13:J14"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="N13:N14"/>
-    <mergeCell ref="O13:O14"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H11:I12"/>
-    <mergeCell ref="C11:D12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H9:I10"/>
-    <mergeCell ref="C9:D10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="H7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="N7:N8"/>
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="E2:G3"/>
-    <mergeCell ref="I2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:O3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="C7:D8"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="L5:L6"/>
-    <mergeCell ref="N5:N6"/>
-    <mergeCell ref="O5:O6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.31496062992125984" right="0.31496062992125984" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
fix(template): update overtime template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/overtime_template.xlsx
+++ b/public/templates/overtime_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\dev\projects\wordtoexcel\staff_manager\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{096AEEDD-236E-419A-A7CB-845CF0377440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2653DDDB-F391-4018-9F2C-C2385A418923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1440" yWindow="1365" windowWidth="28455" windowHeight="18705" xr2:uid="{63E1F611-5DC4-40BF-8CF5-995E8AE1ECB1}"/>
   </bookViews>
@@ -206,7 +206,7 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>{{rest_check_n}}補休     時</t>
+    <t>{{rest_check_n}}補休    時</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>

</xml_diff>